<commit_message>
Replace one-day visit Excel template
</commit_message>
<xml_diff>
--- a/template/cfs_one_day.xlsx
+++ b/template/cfs_one_day.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hansunggroup-my.sharepoint.com/personal/kkmm99jj_hs100_co_kr/Documents/바탕 화면/출입신청/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kkmm99jj/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="711" documentId="8_{C7839102-48C4-4B4B-BACB-F82AED610C1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5611208C-C4C5-46B4-BAD8-087134F2992B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B08E9515-423F-5F49-B9FA-51FA58DA2386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31635" yWindow="2835" windowWidth="17280" windowHeight="11040" xr2:uid="{EF6E6FAA-5F72-459F-97EC-2666CDFDC51B}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" xr2:uid="{EF6E6FAA-5F72-459F-97EC-2666CDFDC51B}"/>
   </bookViews>
   <sheets>
     <sheet name="단체 출입 신청서" sheetId="1" r:id="rId1"/>
@@ -149,10 +149,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="176" formatCode="m&quot;/&quot;d\ \(aaa\)"/>
+    <numFmt numFmtId="176" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="177" formatCode="m&quot;/&quot;d\ \(aaa\)"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -456,7 +456,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -524,10 +524,10 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="8" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="41" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -548,24 +548,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -587,9 +569,18 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -600,6 +591,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -976,54 +976,54 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AF127"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
-    <col min="1" max="1" width="2.19921875" customWidth="1"/>
-    <col min="2" max="2" width="3.796875" customWidth="1"/>
-    <col min="3" max="3" width="12.8984375" customWidth="1"/>
-    <col min="4" max="4" width="15.296875" customWidth="1"/>
-    <col min="5" max="5" width="17.69921875" customWidth="1"/>
-    <col min="6" max="6" width="14.19921875" customWidth="1"/>
+    <col min="1" max="1" width="2.1640625" customWidth="1"/>
+    <col min="2" max="2" width="3.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" customWidth="1"/>
+    <col min="5" max="5" width="17.6640625" customWidth="1"/>
+    <col min="6" max="6" width="14.1640625" customWidth="1"/>
     <col min="7" max="7" width="12.5" customWidth="1"/>
-    <col min="8" max="8" width="7.8984375" customWidth="1"/>
+    <col min="8" max="8" width="7.83203125" customWidth="1"/>
     <col min="9" max="9" width="8" customWidth="1"/>
     <col min="10" max="10" width="11" customWidth="1"/>
     <col min="11" max="11" width="9.5" customWidth="1"/>
-    <col min="12" max="12" width="3.09765625" customWidth="1"/>
-    <col min="13" max="32" width="8.8984375" style="3"/>
+    <col min="12" max="12" width="3.1640625" customWidth="1"/>
+    <col min="13" max="32" width="8.83203125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="10.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:13" ht="11" customHeight="1">
+      <c r="A1" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
-      <c r="K1" s="34"/>
-      <c r="L1" s="34"/>
-    </row>
-    <row r="2" spans="1:13" ht="39.6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="34"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
-      <c r="K2" s="34"/>
-      <c r="L2" s="34"/>
-    </row>
-    <row r="3" spans="1:13" ht="4.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
+    </row>
+    <row r="2" spans="1:13" ht="39.5" customHeight="1">
+      <c r="A2" s="46"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+      <c r="J2" s="46"/>
+      <c r="K2" s="46"/>
+      <c r="L2" s="46"/>
+    </row>
+    <row r="3" spans="1:13" ht="4.25" customHeight="1">
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -1036,28 +1036,28 @@
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
     </row>
-    <row r="4" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="29" t="s">
+    <row r="4" spans="1:13" ht="20.75" customHeight="1">
+      <c r="B4" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="29"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
       <c r="F4" s="10"/>
       <c r="G4" s="10"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="36"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="36"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="29" t="s">
+    <row r="5" spans="1:13" ht="20.75" customHeight="1">
+      <c r="B5" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="29"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
       <c r="F5" s="10"/>
       <c r="G5" s="10"/>
       <c r="H5" s="26"/>
@@ -1066,61 +1066,61 @@
       <c r="K5" s="26"/>
       <c r="L5" s="2"/>
     </row>
-    <row r="6" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="29" t="s">
+    <row r="6" spans="1:13" ht="20.75" customHeight="1">
+      <c r="B6" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="29"/>
-      <c r="D6" s="46"/>
-      <c r="E6" s="46"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="43"/>
       <c r="F6" s="11"/>
       <c r="G6" s="11"/>
-      <c r="H6" s="37"/>
-      <c r="I6" s="37"/>
-      <c r="J6" s="37"/>
-      <c r="K6" s="37"/>
-    </row>
-    <row r="7" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="31"/>
-      <c r="C7" s="31"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
+      <c r="J6" s="31"/>
+      <c r="K6" s="31"/>
+    </row>
+    <row r="7" spans="1:13" ht="20.75" customHeight="1">
+      <c r="B7" s="44"/>
+      <c r="C7" s="44"/>
       <c r="D7" s="7"/>
       <c r="E7" s="28"/>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
-      <c r="H7" s="38" t="s">
+      <c r="H7" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="I7" s="39"/>
-      <c r="J7" s="39"/>
-      <c r="K7" s="39"/>
-    </row>
-    <row r="8" spans="1:13" ht="8.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="33"/>
-      <c r="J8" s="33"/>
-      <c r="K8" s="33"/>
-    </row>
-    <row r="9" spans="1:13" ht="36" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B9" s="43" t="s">
+      <c r="I7" s="33"/>
+      <c r="J7" s="33"/>
+      <c r="K7" s="33"/>
+    </row>
+    <row r="8" spans="1:13" ht="8.75" customHeight="1" thickBot="1">
+      <c r="B8" s="45"/>
+      <c r="C8" s="45"/>
+      <c r="D8" s="45"/>
+      <c r="E8" s="45"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="45"/>
+      <c r="H8" s="45"/>
+      <c r="I8" s="45"/>
+      <c r="J8" s="45"/>
+      <c r="K8" s="45"/>
+    </row>
+    <row r="9" spans="1:13" ht="36" customHeight="1" thickTop="1" thickBot="1">
+      <c r="B9" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="44"/>
-      <c r="D9" s="45"/>
-      <c r="E9" s="45"/>
-      <c r="F9" s="45"/>
-      <c r="G9" s="45"/>
-      <c r="H9" s="45"/>
-      <c r="I9" s="45"/>
-      <c r="J9" s="45"/>
-      <c r="K9" s="45"/>
-    </row>
-    <row r="10" spans="1:13" ht="4.2" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
+      <c r="C9" s="41"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="42"/>
+      <c r="H9" s="42"/>
+      <c r="I9" s="42"/>
+      <c r="J9" s="42"/>
+      <c r="K9" s="42"/>
+    </row>
+    <row r="10" spans="1:13" ht="4.25" customHeight="1" thickTop="1">
       <c r="B10" s="6"/>
       <c r="C10" s="7"/>
       <c r="D10" s="8"/>
@@ -1132,7 +1132,7 @@
       <c r="J10" s="8"/>
       <c r="K10" s="8"/>
     </row>
-    <row r="11" spans="1:13" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:13" ht="20.5" customHeight="1">
       <c r="B11" s="6"/>
       <c r="C11" s="7"/>
       <c r="D11" s="8"/>
@@ -1146,7 +1146,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="8"/>
     </row>
-    <row r="12" spans="1:13" ht="36.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:13" ht="36.75" customHeight="1">
       <c r="B12" s="17" t="s">
         <v>2</v>
       </c>
@@ -1168,13 +1168,13 @@
       <c r="H12" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="I12" s="42" t="s">
+      <c r="I12" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="J12" s="29"/>
-      <c r="K12" s="29"/>
-    </row>
-    <row r="13" spans="1:13" ht="31.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="J12" s="38"/>
+      <c r="K12" s="38"/>
+    </row>
+    <row r="13" spans="1:13" ht="32" customHeight="1">
       <c r="B13" s="19">
         <v>1</v>
       </c>
@@ -1184,12 +1184,12 @@
       <c r="F13" s="25"/>
       <c r="G13" s="21"/>
       <c r="H13" s="22"/>
-      <c r="I13" s="30"/>
-      <c r="J13" s="30"/>
-      <c r="K13" s="30"/>
+      <c r="I13" s="39"/>
+      <c r="J13" s="39"/>
+      <c r="K13" s="39"/>
       <c r="M13" s="9"/>
     </row>
-    <row r="14" spans="1:13" ht="31.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:13" ht="32" customHeight="1">
       <c r="B14" s="19">
         <v>2</v>
       </c>
@@ -1199,12 +1199,12 @@
       <c r="F14" s="25"/>
       <c r="G14" s="21"/>
       <c r="H14" s="22"/>
-      <c r="I14" s="30"/>
-      <c r="J14" s="30"/>
-      <c r="K14" s="30"/>
+      <c r="I14" s="39"/>
+      <c r="J14" s="39"/>
+      <c r="K14" s="39"/>
       <c r="M14" s="9"/>
     </row>
-    <row r="15" spans="1:13" ht="31.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:13" ht="32" customHeight="1">
       <c r="B15" s="19">
         <v>3</v>
       </c>
@@ -1214,12 +1214,12 @@
       <c r="F15" s="25"/>
       <c r="G15" s="21"/>
       <c r="H15" s="22"/>
-      <c r="I15" s="30"/>
-      <c r="J15" s="30"/>
-      <c r="K15" s="30"/>
+      <c r="I15" s="39"/>
+      <c r="J15" s="39"/>
+      <c r="K15" s="39"/>
       <c r="M15" s="9"/>
     </row>
-    <row r="16" spans="1:13" ht="31.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:13" ht="32" customHeight="1">
       <c r="B16" s="19">
         <v>4</v>
       </c>
@@ -1229,12 +1229,12 @@
       <c r="F16" s="25"/>
       <c r="G16" s="21"/>
       <c r="H16" s="22"/>
-      <c r="I16" s="30"/>
-      <c r="J16" s="30"/>
-      <c r="K16" s="30"/>
+      <c r="I16" s="39"/>
+      <c r="J16" s="39"/>
+      <c r="K16" s="39"/>
       <c r="M16" s="9"/>
     </row>
-    <row r="17" spans="2:13" ht="31.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:13" ht="32" customHeight="1">
       <c r="B17" s="19">
         <v>5</v>
       </c>
@@ -1244,12 +1244,12 @@
       <c r="F17" s="25"/>
       <c r="G17" s="21"/>
       <c r="H17" s="22"/>
-      <c r="I17" s="30"/>
-      <c r="J17" s="30"/>
-      <c r="K17" s="30"/>
+      <c r="I17" s="39"/>
+      <c r="J17" s="39"/>
+      <c r="K17" s="39"/>
       <c r="M17" s="9"/>
     </row>
-    <row r="18" spans="2:13" ht="31.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:13" ht="32" customHeight="1">
       <c r="B18" s="19">
         <v>6</v>
       </c>
@@ -1259,12 +1259,12 @@
       <c r="F18" s="25"/>
       <c r="G18" s="21"/>
       <c r="H18" s="22"/>
-      <c r="I18" s="30"/>
-      <c r="J18" s="30"/>
-      <c r="K18" s="30"/>
+      <c r="I18" s="39"/>
+      <c r="J18" s="39"/>
+      <c r="K18" s="39"/>
       <c r="M18" s="9"/>
     </row>
-    <row r="19" spans="2:13" ht="31.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:13" ht="32" customHeight="1">
       <c r="B19" s="19">
         <v>7</v>
       </c>
@@ -1274,12 +1274,12 @@
       <c r="F19" s="25"/>
       <c r="G19" s="21"/>
       <c r="H19" s="22"/>
-      <c r="I19" s="30"/>
-      <c r="J19" s="30"/>
-      <c r="K19" s="30"/>
+      <c r="I19" s="39"/>
+      <c r="J19" s="39"/>
+      <c r="K19" s="39"/>
       <c r="M19" s="9"/>
     </row>
-    <row r="20" spans="2:13" ht="31.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:13" ht="32" customHeight="1">
       <c r="B20" s="19">
         <v>8</v>
       </c>
@@ -1289,12 +1289,12 @@
       <c r="F20" s="25"/>
       <c r="G20" s="21"/>
       <c r="H20" s="22"/>
-      <c r="I20" s="30"/>
-      <c r="J20" s="30"/>
-      <c r="K20" s="30"/>
+      <c r="I20" s="39"/>
+      <c r="J20" s="39"/>
+      <c r="K20" s="39"/>
       <c r="M20" s="9"/>
     </row>
-    <row r="21" spans="2:13" ht="31.95" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="2:13" ht="32" customHeight="1">
       <c r="B21" s="19">
         <v>9</v>
       </c>
@@ -1304,12 +1304,12 @@
       <c r="F21" s="24"/>
       <c r="G21" s="21"/>
       <c r="H21" s="22"/>
-      <c r="I21" s="30"/>
-      <c r="J21" s="30"/>
-      <c r="K21" s="30"/>
+      <c r="I21" s="39"/>
+      <c r="J21" s="39"/>
+      <c r="K21" s="39"/>
       <c r="M21" s="9"/>
     </row>
-    <row r="22" spans="2:13" ht="31.95" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="2:13" ht="32" customHeight="1">
       <c r="B22" s="19">
         <v>10</v>
       </c>
@@ -1319,12 +1319,12 @@
       <c r="F22" s="24"/>
       <c r="G22" s="21"/>
       <c r="H22" s="22"/>
-      <c r="I22" s="30"/>
-      <c r="J22" s="30"/>
-      <c r="K22" s="30"/>
+      <c r="I22" s="39"/>
+      <c r="J22" s="39"/>
+      <c r="K22" s="39"/>
       <c r="M22" s="9"/>
     </row>
-    <row r="23" spans="2:13" ht="31.2" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="2:13" ht="32" customHeight="1">
       <c r="B23" s="19">
         <v>11</v>
       </c>
@@ -1334,12 +1334,12 @@
       <c r="F23" s="24"/>
       <c r="G23" s="21"/>
       <c r="H23" s="22"/>
-      <c r="I23" s="30"/>
-      <c r="J23" s="30"/>
-      <c r="K23" s="30"/>
+      <c r="I23" s="39"/>
+      <c r="J23" s="39"/>
+      <c r="K23" s="39"/>
       <c r="M23" s="9"/>
     </row>
-    <row r="24" spans="2:13" ht="31.95" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="2:13" ht="32" customHeight="1">
       <c r="B24" s="19">
         <v>12</v>
       </c>
@@ -1349,14 +1349,14 @@
       <c r="F24" s="24"/>
       <c r="G24" s="21"/>
       <c r="H24" s="22"/>
-      <c r="I24" s="30"/>
-      <c r="J24" s="30"/>
-      <c r="K24" s="30"/>
+      <c r="I24" s="39"/>
+      <c r="J24" s="39"/>
+      <c r="K24" s="39"/>
       <c r="M24" s="9" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="2:13" ht="31.95" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="2:13" ht="57" hidden="1" customHeight="1">
       <c r="B25" s="19">
         <v>13</v>
       </c>
@@ -1366,12 +1366,12 @@
       <c r="F25" s="24"/>
       <c r="G25" s="21"/>
       <c r="H25" s="22"/>
-      <c r="I25" s="30"/>
-      <c r="J25" s="30"/>
-      <c r="K25" s="30"/>
+      <c r="I25" s="39"/>
+      <c r="J25" s="39"/>
+      <c r="K25" s="39"/>
       <c r="M25" s="4"/>
     </row>
-    <row r="26" spans="2:13" ht="31.95" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="2:13" ht="77" hidden="1" customHeight="1">
       <c r="B26" s="19">
         <v>14</v>
       </c>
@@ -1381,12 +1381,12 @@
       <c r="F26" s="24"/>
       <c r="G26" s="21"/>
       <c r="H26" s="22"/>
-      <c r="I26" s="30"/>
-      <c r="J26" s="30"/>
-      <c r="K26" s="30"/>
+      <c r="I26" s="39"/>
+      <c r="J26" s="39"/>
+      <c r="K26" s="39"/>
       <c r="M26" s="4"/>
     </row>
-    <row r="27" spans="2:13" ht="31.95" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="2:13" ht="16" hidden="1" customHeight="1">
       <c r="B27" s="19">
         <v>15</v>
       </c>
@@ -1396,144 +1396,161 @@
       <c r="F27" s="24"/>
       <c r="G27" s="21"/>
       <c r="H27" s="22"/>
-      <c r="I27" s="30"/>
-      <c r="J27" s="30"/>
-      <c r="K27" s="30"/>
+      <c r="I27" s="39"/>
+      <c r="J27" s="39"/>
+      <c r="K27" s="39"/>
       <c r="M27" s="4"/>
     </row>
-    <row r="28" spans="2:13" ht="21.15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B28" s="29" t="s">
+    <row r="28" spans="2:13" ht="21.25" customHeight="1">
+      <c r="B28" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="C28" s="29"/>
-      <c r="D28" s="29"/>
-      <c r="E28" s="29"/>
-      <c r="F28" s="40" t="s">
+      <c r="C28" s="38"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="G28" s="40"/>
-      <c r="H28" s="40"/>
-      <c r="I28" s="40"/>
-      <c r="J28" s="40"/>
-      <c r="K28" s="40"/>
-    </row>
-    <row r="29" spans="2:13" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B29" s="35"/>
-      <c r="C29" s="35"/>
-      <c r="D29" s="35"/>
-      <c r="E29" s="35"/>
-      <c r="F29" s="41" t="s">
+      <c r="G28" s="34"/>
+      <c r="H28" s="34"/>
+      <c r="I28" s="34"/>
+      <c r="J28" s="34"/>
+      <c r="K28" s="34"/>
+    </row>
+    <row r="29" spans="2:13" ht="40.25" customHeight="1">
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="G29" s="41"/>
-      <c r="H29" s="41"/>
-      <c r="I29" s="41"/>
-      <c r="J29" s="41"/>
-      <c r="K29" s="41"/>
+      <c r="G29" s="35"/>
+      <c r="H29" s="35"/>
+      <c r="I29" s="35"/>
+      <c r="J29" s="35"/>
+      <c r="K29" s="35"/>
       <c r="M29" s="5"/>
     </row>
-    <row r="30" spans="2:13" ht="45.6" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="2:13" ht="45.5" customHeight="1">
       <c r="K30" s="16"/>
     </row>
-    <row r="31" spans="2:13" s="3" customFormat="1" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="32" spans="2:13" s="3" customFormat="1" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="33" s="3" customFormat="1" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="34" s="3" customFormat="1" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="35" s="3" customFormat="1" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="36" s="3" customFormat="1" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="37" s="3" customFormat="1" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="38" s="3" customFormat="1" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="39" s="3" customFormat="1" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="40" s="3" customFormat="1" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="41" s="3" customFormat="1" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="42" s="3" customFormat="1" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="43" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="44" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="45" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="46" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="47" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="48" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="49" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="50" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="51" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="52" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="53" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="54" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="55" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="56" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="57" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="58" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="59" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="60" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="61" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="62" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="63" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="64" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="65" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="66" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="67" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="68" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="69" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="70" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="71" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="72" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="73" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="74" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="75" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="76" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="77" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="78" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="79" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="80" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="81" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="82" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="83" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="84" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="85" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="86" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="87" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="88" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="89" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="90" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="91" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="92" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="93" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="94" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="95" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="96" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="97" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="98" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="99" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="100" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="101" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="102" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="103" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="104" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="105" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="106" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="107" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="108" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="109" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="110" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="111" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="112" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="113" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="114" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="115" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="116" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="117" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="118" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="119" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="120" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="121" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="122" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="123" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="124" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="125" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="126" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="127" s="3" customFormat="1" x14ac:dyDescent="0.4"/>
+    <row r="31" spans="2:13" s="3" customFormat="1" ht="66.5" customHeight="1"/>
+    <row r="32" spans="2:13" s="3" customFormat="1" ht="66.5" customHeight="1"/>
+    <row r="33" s="3" customFormat="1" ht="66.5" customHeight="1"/>
+    <row r="34" s="3" customFormat="1" ht="66.5" customHeight="1"/>
+    <row r="35" s="3" customFormat="1" ht="66.5" customHeight="1"/>
+    <row r="36" s="3" customFormat="1" ht="66.5" customHeight="1"/>
+    <row r="37" s="3" customFormat="1" ht="66.5" customHeight="1"/>
+    <row r="38" s="3" customFormat="1" ht="66.5" customHeight="1"/>
+    <row r="39" s="3" customFormat="1" ht="66.5" customHeight="1"/>
+    <row r="40" s="3" customFormat="1" ht="66.5" customHeight="1"/>
+    <row r="41" s="3" customFormat="1" ht="66.5" customHeight="1"/>
+    <row r="42" s="3" customFormat="1" ht="66.5" customHeight="1"/>
+    <row r="43" s="3" customFormat="1"/>
+    <row r="44" s="3" customFormat="1"/>
+    <row r="45" s="3" customFormat="1"/>
+    <row r="46" s="3" customFormat="1"/>
+    <row r="47" s="3" customFormat="1"/>
+    <row r="48" s="3" customFormat="1"/>
+    <row r="49" s="3" customFormat="1"/>
+    <row r="50" s="3" customFormat="1"/>
+    <row r="51" s="3" customFormat="1"/>
+    <row r="52" s="3" customFormat="1"/>
+    <row r="53" s="3" customFormat="1"/>
+    <row r="54" s="3" customFormat="1"/>
+    <row r="55" s="3" customFormat="1"/>
+    <row r="56" s="3" customFormat="1"/>
+    <row r="57" s="3" customFormat="1"/>
+    <row r="58" s="3" customFormat="1"/>
+    <row r="59" s="3" customFormat="1"/>
+    <row r="60" s="3" customFormat="1"/>
+    <row r="61" s="3" customFormat="1"/>
+    <row r="62" s="3" customFormat="1"/>
+    <row r="63" s="3" customFormat="1"/>
+    <row r="64" s="3" customFormat="1"/>
+    <row r="65" s="3" customFormat="1"/>
+    <row r="66" s="3" customFormat="1"/>
+    <row r="67" s="3" customFormat="1"/>
+    <row r="68" s="3" customFormat="1"/>
+    <row r="69" s="3" customFormat="1"/>
+    <row r="70" s="3" customFormat="1"/>
+    <row r="71" s="3" customFormat="1"/>
+    <row r="72" s="3" customFormat="1"/>
+    <row r="73" s="3" customFormat="1"/>
+    <row r="74" s="3" customFormat="1"/>
+    <row r="75" s="3" customFormat="1"/>
+    <row r="76" s="3" customFormat="1"/>
+    <row r="77" s="3" customFormat="1"/>
+    <row r="78" s="3" customFormat="1"/>
+    <row r="79" s="3" customFormat="1"/>
+    <row r="80" s="3" customFormat="1"/>
+    <row r="81" s="3" customFormat="1"/>
+    <row r="82" s="3" customFormat="1"/>
+    <row r="83" s="3" customFormat="1"/>
+    <row r="84" s="3" customFormat="1"/>
+    <row r="85" s="3" customFormat="1"/>
+    <row r="86" s="3" customFormat="1"/>
+    <row r="87" s="3" customFormat="1"/>
+    <row r="88" s="3" customFormat="1"/>
+    <row r="89" s="3" customFormat="1"/>
+    <row r="90" s="3" customFormat="1"/>
+    <row r="91" s="3" customFormat="1"/>
+    <row r="92" s="3" customFormat="1"/>
+    <row r="93" s="3" customFormat="1"/>
+    <row r="94" s="3" customFormat="1"/>
+    <row r="95" s="3" customFormat="1"/>
+    <row r="96" s="3" customFormat="1"/>
+    <row r="97" s="3" customFormat="1"/>
+    <row r="98" s="3" customFormat="1"/>
+    <row r="99" s="3" customFormat="1"/>
+    <row r="100" s="3" customFormat="1"/>
+    <row r="101" s="3" customFormat="1"/>
+    <row r="102" s="3" customFormat="1"/>
+    <row r="103" s="3" customFormat="1"/>
+    <row r="104" s="3" customFormat="1"/>
+    <row r="105" s="3" customFormat="1"/>
+    <row r="106" s="3" customFormat="1"/>
+    <row r="107" s="3" customFormat="1"/>
+    <row r="108" s="3" customFormat="1"/>
+    <row r="109" s="3" customFormat="1"/>
+    <row r="110" s="3" customFormat="1"/>
+    <row r="111" s="3" customFormat="1"/>
+    <row r="112" s="3" customFormat="1"/>
+    <row r="113" s="3" customFormat="1"/>
+    <row r="114" s="3" customFormat="1"/>
+    <row r="115" s="3" customFormat="1"/>
+    <row r="116" s="3" customFormat="1"/>
+    <row r="117" s="3" customFormat="1"/>
+    <row r="118" s="3" customFormat="1"/>
+    <row r="119" s="3" customFormat="1"/>
+    <row r="120" s="3" customFormat="1"/>
+    <row r="121" s="3" customFormat="1"/>
+    <row r="122" s="3" customFormat="1"/>
+    <row r="123" s="3" customFormat="1"/>
+    <row r="124" s="3" customFormat="1"/>
+    <row r="125" s="3" customFormat="1"/>
+    <row r="126" s="3" customFormat="1"/>
+    <row r="127" s="3" customFormat="1"/>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="I23:K23"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="B8:K8"/>
+    <mergeCell ref="A1:L2"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="I25:K25"/>
+    <mergeCell ref="I24:K24"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="I15:K15"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="I18:K18"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="I22:K22"/>
     <mergeCell ref="B29:E29"/>
     <mergeCell ref="H4:K4"/>
     <mergeCell ref="H6:K6"/>
@@ -1550,23 +1567,6 @@
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="B8:K8"/>
-    <mergeCell ref="A1:L2"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="I25:K25"/>
-    <mergeCell ref="I24:K24"/>
-    <mergeCell ref="I14:K14"/>
-    <mergeCell ref="I15:K15"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="I22:K22"/>
-    <mergeCell ref="I23:K23"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="1">
@@ -1584,17 +1584,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5884e97d-3119-4664-b9fd-3d8a26201c4b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="6b0c99c4-3b86-43f4-a675-1126333bd00d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<titus xmlns="http://schemas.titus.com/TitusProperties/">
+  <TitusGUID xmlns="">732ab167-7550-414f-8032-c71fcd84de0a</TitusGUID>
+</titus>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DCAED1A0B5520B439D6DAF46938781B4" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a8c86e330b5f1d48d59a3d8067facbc7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5884e97d-3119-4664-b9fd-3d8a26201c4b" xmlns:ns3="6b0c99c4-3b86-43f4-a675-1126333bd00d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d434fab2495591418147bb6a556859ca" ns2:_="" ns3:_="">
     <xsd:import namespace="5884e97d-3119-4664-b9fd-3d8a26201c4b"/>
@@ -1829,35 +1833,35 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<titus xmlns="http://schemas.titus.com/TitusProperties/">
-  <TitusGUID xmlns="">732ab167-7550-414f-8032-c71fcd84de0a</TitusGUID>
-</titus>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5884e97d-3119-4664-b9fd-3d8a26201c4b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="6b0c99c4-3b86-43f4-a675-1126333bd00d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{92D8EEA2-79F4-46A9-8FC4-8C4033121860}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3EA9131F-27D7-4344-A58E-48417B5B946A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2000/xmlns/"/>
-    <ds:schemaRef ds:uri="5884e97d-3119-4664-b9fd-3d8a26201c4b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6b0c99c4-3b86-43f4-a675-1126333bd00d"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema-instance"/>
+    <ds:schemaRef ds:uri="http://schemas.titus.com/TitusProperties/"/>
+    <ds:schemaRef ds:uri=""/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38685B65-56A2-4CBC-A29B-BBC67238597F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BC1F21C-687C-49CB-AAB8-1047B86CEF6E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1877,19 +1881,15 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38685B65-56A2-4CBC-A29B-BBC67238597F}">
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{92D8EEA2-79F4-46A9-8FC4-8C4033121860}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3EA9131F-27D7-4344-A58E-48417B5B946A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.titus.com/TitusProperties/"/>
-    <ds:schemaRef ds:uri=""/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2000/xmlns/"/>
+    <ds:schemaRef ds:uri="5884e97d-3119-4664-b9fd-3d8a26201c4b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6b0c99c4-3b86-43f4-a675-1126333bd00d"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema-instance"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>